<commit_message>
Push all project files to GitHub
</commit_message>
<xml_diff>
--- a/data/alerts.xlsx
+++ b/data/alerts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,6 +458,36 @@
         <is>
           <t>is_read</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>110387d4-f1fa-4fad-8084-96bbceccb8f5</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>6a9169d9-2385-49fc-a24a-99b8eb9437e8</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>welcome</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Welcome to CropMonitor! Start by adding your first crop.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2025-04-15 14:42:17</t>
+        </is>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>